<commit_message>
Did a lot of work on the proliferation growth curves; did a minimum number of points, highligting exp. phase, etc.
</commit_message>
<xml_diff>
--- a/proliferation_growth_curves/Incucyte_sheets/r6.xlsx
+++ b/proliferation_growth_curves/Incucyte_sheets/r6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allielas/HTP_fibroblasts_mitolyso/proliferation_growth_curves/Incucyte_sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBD0C0CE-8151-224C-BEA4-5D7715C1B537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDFCDE5E-5A58-E94D-915B-4BCD599A61F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38940" yWindow="1220" windowWidth="38080" windowHeight="20780" xr2:uid="{7BEA321C-1B3D-3246-BC4D-25D7711379CE}"/>
+    <workbookView xWindow="-38400" yWindow="-4460" windowWidth="38080" windowHeight="20780" xr2:uid="{7BEA321C-1B3D-3246-BC4D-25D7711379CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Reformatted" sheetId="3" r:id="rId1"/>
@@ -591,9 +591,6 @@
     <t>Vessel Name: 20250410_AS_MRC5_Confluence_Rep6_Plate2</t>
   </si>
   <si>
-    <t>Vessel Name</t>
-  </si>
-  <si>
     <t>20250410_AS_MRC5_Confluence_Rep6</t>
   </si>
   <si>
@@ -1138,6 +1135,9 @@
   </si>
   <si>
     <t>P13 LIN12-0C-b2-s2 (B4), Image 9</t>
+  </si>
+  <si>
+    <t>Vessel_Name</t>
   </si>
 </sst>
 </file>
@@ -2060,553 +2060,553 @@
   <sheetData>
     <row r="1" spans="1:183" s="5" customFormat="1" ht="85" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>189</v>
+        <v>371</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="W1" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="Z1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AB1" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AC1" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="AD1" s="6" t="s">
+      <c r="AE1" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AF1" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="AF1" s="6" t="s">
+      <c r="AG1" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="AG1" s="6" t="s">
+      <c r="AH1" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="AH1" s="6" t="s">
+      <c r="AI1" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="AI1" s="6" t="s">
+      <c r="AJ1" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="AJ1" s="6" t="s">
+      <c r="AK1" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="AK1" s="6" t="s">
+      <c r="AL1" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="AL1" s="6" t="s">
+      <c r="AM1" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="AM1" s="6" t="s">
+      <c r="AN1" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="AN1" s="6" t="s">
+      <c r="AO1" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="AO1" s="6" t="s">
+      <c r="AP1" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="AP1" s="6" t="s">
+      <c r="AQ1" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="AQ1" s="6" t="s">
+      <c r="AR1" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="AR1" s="6" t="s">
+      <c r="AS1" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="AS1" s="6" t="s">
+      <c r="AT1" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="AT1" s="6" t="s">
+      <c r="AU1" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="AU1" s="6" t="s">
+      <c r="AV1" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="AV1" s="6" t="s">
+      <c r="AW1" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="AW1" s="6" t="s">
+      <c r="AX1" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="AX1" s="6" t="s">
+      <c r="AY1" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="AY1" s="6" t="s">
+      <c r="AZ1" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="AZ1" s="6" t="s">
+      <c r="BA1" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="BA1" s="6" t="s">
+      <c r="BB1" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="BB1" s="6" t="s">
+      <c r="BC1" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="BC1" s="6" t="s">
+      <c r="BD1" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="BD1" s="6" t="s">
+      <c r="BE1" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="BE1" s="6" t="s">
+      <c r="BF1" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="BF1" s="6" t="s">
+      <c r="BG1" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="BG1" s="6" t="s">
+      <c r="BH1" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="BH1" s="6" t="s">
+      <c r="BI1" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="BI1" s="6" t="s">
+      <c r="BJ1" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="BJ1" s="6" t="s">
+      <c r="BK1" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="BK1" s="6" t="s">
+      <c r="BL1" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="BL1" s="6" t="s">
+      <c r="BM1" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="BM1" s="6" t="s">
+      <c r="BN1" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="BN1" s="6" t="s">
+      <c r="BO1" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="BO1" s="6" t="s">
+      <c r="BP1" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="BP1" s="6" t="s">
+      <c r="BQ1" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="BQ1" s="6" t="s">
+      <c r="BR1" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="BR1" s="6" t="s">
+      <c r="BS1" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="BS1" s="6" t="s">
+      <c r="BT1" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="BT1" s="6" t="s">
+      <c r="BU1" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="BU1" s="6" t="s">
+      <c r="BV1" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="BV1" s="6" t="s">
+      <c r="BW1" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="BW1" s="6" t="s">
+      <c r="BX1" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="BX1" s="6" t="s">
+      <c r="BY1" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="BY1" s="6" t="s">
+      <c r="BZ1" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="BZ1" s="6" t="s">
+      <c r="CA1" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="CA1" s="6" t="s">
+      <c r="CB1" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="CB1" s="6" t="s">
+      <c r="CC1" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="CC1" s="6" t="s">
+      <c r="CD1" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="CD1" s="6" t="s">
+      <c r="CE1" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="CE1" s="6" t="s">
+      <c r="CF1" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="CF1" s="6" t="s">
+      <c r="CG1" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="CG1" s="6" t="s">
+      <c r="CH1" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="CH1" s="6" t="s">
+      <c r="CI1" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="CI1" s="6" t="s">
+      <c r="CJ1" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="CJ1" s="6" t="s">
+      <c r="CK1" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="CK1" s="6" t="s">
+      <c r="CL1" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="CL1" s="6" t="s">
+      <c r="CM1" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="CM1" s="6" t="s">
+      <c r="CN1" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="CN1" s="6" t="s">
+      <c r="CO1" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="CO1" s="6" t="s">
+      <c r="CP1" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="CP1" s="6" t="s">
+      <c r="CQ1" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="CQ1" s="6" t="s">
+      <c r="CR1" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="CR1" s="6" t="s">
+      <c r="CS1" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="CS1" s="6" t="s">
+      <c r="CT1" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="CT1" s="6" t="s">
+      <c r="CU1" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="CU1" s="6" t="s">
+      <c r="CV1" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="CV1" s="6" t="s">
+      <c r="CW1" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="CW1" s="6" t="s">
+      <c r="CX1" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="CX1" s="6" t="s">
+      <c r="CY1" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="CY1" s="6" t="s">
+      <c r="CZ1" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="CZ1" s="6" t="s">
+      <c r="DA1" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="DA1" s="6" t="s">
+      <c r="DB1" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="DB1" s="6" t="s">
+      <c r="DC1" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="DC1" s="6" t="s">
+      <c r="DD1" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="DD1" s="6" t="s">
+      <c r="DE1" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="DE1" s="6" t="s">
+      <c r="DF1" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="DF1" s="6" t="s">
+      <c r="DG1" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="DG1" s="6" t="s">
+      <c r="DH1" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="DH1" s="6" t="s">
+      <c r="DI1" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="DI1" s="6" t="s">
+      <c r="DJ1" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="DJ1" s="6" t="s">
+      <c r="DK1" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="DK1" s="6" t="s">
+      <c r="DL1" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="DL1" s="6" t="s">
+      <c r="DM1" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="DM1" s="6" t="s">
+      <c r="DN1" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="DN1" s="6" t="s">
+      <c r="DO1" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="DO1" s="6" t="s">
+      <c r="DP1" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="DP1" s="6" t="s">
+      <c r="DQ1" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="DQ1" s="6" t="s">
+      <c r="DR1" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="DR1" s="6" t="s">
+      <c r="DS1" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="DS1" s="6" t="s">
+      <c r="DT1" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="DT1" s="6" t="s">
+      <c r="DU1" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="DU1" s="6" t="s">
+      <c r="DV1" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="DV1" s="6" t="s">
+      <c r="DW1" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="DW1" s="6" t="s">
+      <c r="DX1" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="DX1" s="6" t="s">
+      <c r="DY1" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="DY1" s="6" t="s">
+      <c r="DZ1" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="DZ1" s="6" t="s">
+      <c r="EA1" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="EA1" s="6" t="s">
+      <c r="EB1" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="EB1" s="6" t="s">
+      <c r="EC1" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="EC1" s="6" t="s">
+      <c r="ED1" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="ED1" s="6" t="s">
+      <c r="EE1" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="EE1" s="6" t="s">
+      <c r="EF1" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="EF1" s="6" t="s">
+      <c r="EG1" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="EG1" s="6" t="s">
+      <c r="EH1" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="EH1" s="6" t="s">
+      <c r="EI1" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="EI1" s="6" t="s">
+      <c r="EJ1" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="EJ1" s="6" t="s">
+      <c r="EK1" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="EK1" s="6" t="s">
+      <c r="EL1" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="EL1" s="6" t="s">
+      <c r="EM1" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="EM1" s="6" t="s">
+      <c r="EN1" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="EN1" s="6" t="s">
+      <c r="EO1" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="EO1" s="6" t="s">
+      <c r="EP1" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="EP1" s="6" t="s">
+      <c r="EQ1" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="EQ1" s="6" t="s">
+      <c r="ER1" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="ER1" s="6" t="s">
+      <c r="ES1" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="ES1" s="6" t="s">
+      <c r="ET1" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="ET1" s="6" t="s">
+      <c r="EU1" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="EU1" s="6" t="s">
+      <c r="EV1" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="EV1" s="6" t="s">
+      <c r="EW1" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="EW1" s="6" t="s">
+      <c r="EX1" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="EX1" s="6" t="s">
+      <c r="EY1" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="EY1" s="6" t="s">
+      <c r="EZ1" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="EZ1" s="6" t="s">
+      <c r="FA1" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="FA1" s="6" t="s">
+      <c r="FB1" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="FB1" s="6" t="s">
+      <c r="FC1" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="FC1" s="6" t="s">
+      <c r="FD1" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="FD1" s="6" t="s">
+      <c r="FE1" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="FE1" s="6" t="s">
+      <c r="FF1" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="FF1" s="6" t="s">
+      <c r="FG1" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="FG1" s="6" t="s">
+      <c r="FH1" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="FH1" s="6" t="s">
+      <c r="FI1" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="FI1" s="6" t="s">
+      <c r="FJ1" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="FJ1" s="6" t="s">
+      <c r="FK1" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="FK1" s="6" t="s">
+      <c r="FL1" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="FL1" s="6" t="s">
+      <c r="FM1" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="FM1" s="6" t="s">
+      <c r="FN1" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="FN1" s="6" t="s">
+      <c r="FO1" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="FO1" s="6" t="s">
+      <c r="FP1" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="FP1" s="6" t="s">
+      <c r="FQ1" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="FQ1" s="6" t="s">
+      <c r="FR1" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="FR1" s="6" t="s">
+      <c r="FS1" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="FS1" s="6" t="s">
+      <c r="FT1" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="FT1" s="6" t="s">
+      <c r="FU1" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="FU1" s="6" t="s">
+      <c r="FV1" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="FV1" s="6" t="s">
+      <c r="FW1" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="FW1" s="6" t="s">
+      <c r="FX1" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="FX1" s="6" t="s">
+      <c r="FY1" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="FY1" s="6" t="s">
+      <c r="FZ1" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="FZ1" s="6" t="s">
+      <c r="GA1" s="6" t="s">
         <v>370</v>
-      </c>
-      <c r="GA1" s="6" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="2" spans="1:183" x14ac:dyDescent="0.2">
@@ -2614,7 +2614,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C2" s="2">
         <v>0</v>
@@ -3165,7 +3165,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C3" s="2">
         <v>2</v>
@@ -3716,7 +3716,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C4" s="2">
         <v>4</v>
@@ -4267,7 +4267,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C5" s="2">
         <v>6</v>
@@ -4818,7 +4818,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C6" s="2">
         <v>8</v>
@@ -5369,7 +5369,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C7" s="2">
         <v>10</v>
@@ -5920,7 +5920,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C8" s="2">
         <v>12</v>
@@ -6471,7 +6471,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C9" s="2">
         <v>14</v>
@@ -7022,7 +7022,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C10" s="2">
         <v>16</v>
@@ -7573,7 +7573,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C11" s="2">
         <v>18</v>
@@ -8124,7 +8124,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C12" s="2">
         <v>20</v>
@@ -8675,7 +8675,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C13" s="2">
         <v>22</v>
@@ -9226,7 +9226,7 @@
         <v>6</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C14" s="2">
         <v>24</v>
@@ -9777,7 +9777,7 @@
         <v>6</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C15" s="2">
         <v>26</v>
@@ -10328,7 +10328,7 @@
         <v>6</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C16" s="2">
         <v>28</v>
@@ -10879,7 +10879,7 @@
         <v>6</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C17" s="2">
         <v>30</v>
@@ -11430,7 +11430,7 @@
         <v>6</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C18" s="2">
         <v>32</v>
@@ -11981,7 +11981,7 @@
         <v>6</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C19" s="2">
         <v>34</v>
@@ -12532,7 +12532,7 @@
         <v>6</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C20" s="2">
         <v>36</v>
@@ -13083,7 +13083,7 @@
         <v>6</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C21" s="2">
         <v>38</v>
@@ -13634,7 +13634,7 @@
         <v>6</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C22" s="2">
         <v>40</v>
@@ -14185,7 +14185,7 @@
         <v>6</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C23" s="2">
         <v>42</v>
@@ -14736,7 +14736,7 @@
         <v>6</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C24" s="2">
         <v>44</v>
@@ -15287,7 +15287,7 @@
         <v>6</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C25" s="2">
         <v>46</v>
@@ -15838,7 +15838,7 @@
         <v>6</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C26" s="2">
         <v>48</v>
@@ -16389,7 +16389,7 @@
         <v>6</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C27" s="2">
         <v>50</v>
@@ -16940,7 +16940,7 @@
         <v>6</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C28" s="2">
         <v>52</v>
@@ -17491,7 +17491,7 @@
         <v>6</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C29" s="2">
         <v>54</v>
@@ -18042,7 +18042,7 @@
         <v>6</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C30" s="2">
         <v>56</v>
@@ -18593,7 +18593,7 @@
         <v>6</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C31" s="2">
         <v>58</v>
@@ -19144,7 +19144,7 @@
         <v>6</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C32" s="2">
         <v>60</v>
@@ -19695,7 +19695,7 @@
         <v>6</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C33" s="2">
         <v>62</v>
@@ -20246,7 +20246,7 @@
         <v>6</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C34" s="2">
         <v>64</v>
@@ -20797,7 +20797,7 @@
         <v>6</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C35" s="2">
         <v>66</v>
@@ -21348,7 +21348,7 @@
         <v>6</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C36" s="2">
         <v>68</v>
@@ -21899,7 +21899,7 @@
         <v>6</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C37" s="2">
         <v>70</v>
@@ -22450,7 +22450,7 @@
         <v>6</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C38" s="2">
         <v>72</v>

</xml_diff>